<commit_message>
Simplify inspection flow and add scoped reset controls
</commit_message>
<xml_diff>
--- a/data/lekplatskontroll.xlsx
+++ b/data/lekplatskontroll.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{75741EDF-346D-4A1F-AD38-2885EAB38BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{85368D10-49FD-4618-AC34-EE2B75724B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lekplatsmatris" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
   <si>
     <t>Lekplats</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>Gångytan är fri från halkrisk och snubbelrisk</t>
+  </si>
+  <si>
+    <t>Räcken, stolpar och ledstänger är fast förankrade och svajar inte när man lutar sig mot dem.</t>
   </si>
   <si>
     <t>Räcken och skydd sitter stadigt</t>
@@ -1669,7 +1672,7 @@
       <c r="Z5" s="15"/>
       <c r="AA5" s="15"/>
     </row>
-    <row r="6" spans="1:27" s="40" customFormat="1" ht="28.5">
+    <row r="6" spans="1:27" s="40" customFormat="1" ht="72">
       <c r="A6" s="10" t="s">
         <v>19</v>
       </c>
@@ -1706,7 +1709,7 @@
     </row>
     <row r="7" spans="1:27" s="40" customFormat="1" ht="28.5">
       <c r="A7" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>

</xml_diff>

<commit_message>
Fixade bugg i xlsx
</commit_message>
<xml_diff>
--- a/data/lekplatskontroll.xlsx
+++ b/data/lekplatskontroll.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://orebrokommun-my.sharepoint.com/personal/mimmi_beckman_orebro_se/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{082FFA92-712D-4D65-A6DC-D1B3836D4844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1048D69-7278-4DA7-A134-A28402493461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="104">
   <si>
     <t>Lekplats</t>
   </si>
@@ -85,7 +85,7 @@
     <t>Träd</t>
   </si>
   <si>
-    <t>Portaler</t>
+    <t>Portal</t>
   </si>
   <si>
     <t>Lundbyparken</t>
@@ -185,9 +185,6 @@
   </si>
   <si>
     <t>Mariebergs skogslek</t>
-  </si>
-  <si>
-    <t>Portal</t>
   </si>
   <si>
     <t>Fästen för vajrar runt träden är i gott skick.</t>
@@ -2035,7 +2032,7 @@
         <v>14</v>
       </c>
       <c r="O1" s="26" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="P1" s="27"/>
       <c r="Q1" s="27"/>
@@ -2052,49 +2049,49 @@
     </row>
     <row r="2" spans="1:27" s="15" customFormat="1" ht="76.5">
       <c r="A2" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="D2" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="E2" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="F2" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="I2" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="K2" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="L2" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="N2" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="O2" s="29" t="s">
         <v>54</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="I2" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="L2" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="N2" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="O2" s="29" t="s">
-        <v>55</v>
       </c>
       <c r="P2" s="17"/>
       <c r="Q2" s="17"/>
@@ -2111,47 +2108,47 @@
     </row>
     <row r="3" spans="1:27" s="15" customFormat="1" ht="76.5">
       <c r="A3" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="C3" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="D3" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="F3" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="K3" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="I3" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="J3" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="K3" s="20" t="s">
+      <c r="L3" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="M3" s="20" t="s">
         <v>65</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="M3" s="20" t="s">
-        <v>66</v>
       </c>
       <c r="N3" s="30"/>
       <c r="O3" s="30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P3" s="18"/>
       <c r="Q3" s="18"/>
@@ -2168,41 +2165,41 @@
     </row>
     <row r="4" spans="1:27" s="15" customFormat="1" ht="60.75">
       <c r="A4" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="D4" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="E4" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="20" t="s">
-        <v>71</v>
-      </c>
       <c r="F4" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K4" s="20"/>
       <c r="L4" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" s="20" t="s">
         <v>71</v>
-      </c>
-      <c r="M4" s="20" t="s">
-        <v>72</v>
       </c>
       <c r="N4" s="29"/>
       <c r="O4" s="29"/>
@@ -2221,39 +2218,39 @@
     </row>
     <row r="5" spans="1:27" s="15" customFormat="1" ht="76.5">
       <c r="A5" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>73</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>74</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K5" s="23"/>
       <c r="L5" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="M5" s="20" t="s">
         <v>75</v>
-      </c>
-      <c r="M5" s="20" t="s">
-        <v>76</v>
       </c>
       <c r="N5" s="30"/>
       <c r="O5" s="30"/>
@@ -2272,36 +2269,36 @@
     </row>
     <row r="6" spans="1:27" s="15" customFormat="1" ht="60.75">
       <c r="A6" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" s="29"/>
       <c r="D6" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="E6" s="20" t="s">
-        <v>79</v>
-      </c>
       <c r="F6" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K6" s="20"/>
       <c r="L6" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M6" s="29"/>
       <c r="N6" s="29"/>
@@ -2321,18 +2318,18 @@
     </row>
     <row r="7" spans="1:27" s="15" customFormat="1" ht="76.5">
       <c r="A7" s="20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C7" s="30"/>
       <c r="D7" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" s="30"/>
       <c r="F7" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G7" s="30"/>
       <c r="H7" s="30"/>
@@ -2358,16 +2355,16 @@
     </row>
     <row r="8" spans="1:27" s="15" customFormat="1" ht="45.75">
       <c r="A8" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="29"/>
       <c r="D8" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E8" s="29"/>
       <c r="F8" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G8" s="29"/>
       <c r="H8" s="29"/>
@@ -2393,16 +2390,16 @@
     </row>
     <row r="9" spans="1:27" s="15" customFormat="1" ht="76.5">
       <c r="A9" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" s="30"/>
       <c r="C9" s="30"/>
       <c r="D9" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E9" s="30"/>
       <c r="F9" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G9" s="30"/>
       <c r="H9" s="30"/>
@@ -2428,16 +2425,16 @@
     </row>
     <row r="10" spans="1:27" s="15" customFormat="1" ht="30.75">
       <c r="A10" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
       <c r="D10" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E10" s="31"/>
       <c r="F10" s="30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G10" s="31"/>
       <c r="H10" s="31"/>
@@ -2463,16 +2460,16 @@
     </row>
     <row r="11" spans="1:27" s="15" customFormat="1" ht="121.5">
       <c r="A11" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
       <c r="D11" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E11" s="30"/>
       <c r="F11" s="31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="30"/>
@@ -2498,12 +2495,12 @@
     </row>
     <row r="12" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A12" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="21"/>
       <c r="D12" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E12" s="29"/>
       <c r="F12" s="30"/>
@@ -2531,12 +2528,12 @@
     </row>
     <row r="13" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A13" s="20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" s="22"/>
       <c r="C13" s="22"/>
       <c r="D13" s="20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E13" s="30"/>
       <c r="F13" s="29"/>
@@ -2564,12 +2561,12 @@
     </row>
     <row r="14" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A14" s="20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
       <c r="D14" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E14" s="29"/>
       <c r="F14" s="30"/>
@@ -2597,12 +2594,12 @@
     </row>
     <row r="15" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A15" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B15" s="22"/>
       <c r="C15" s="22"/>
       <c r="D15" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E15" s="30"/>
       <c r="F15" s="29"/>
@@ -2630,12 +2627,12 @@
     </row>
     <row r="16" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A16" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29"/>
       <c r="D16" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E16" s="30"/>
       <c r="F16" s="29"/>
@@ -2662,12 +2659,12 @@
     </row>
     <row r="17" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A17" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B17" s="30"/>
       <c r="C17" s="30"/>
       <c r="D17" s="20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" s="30"/>
       <c r="F17" s="29"/>
@@ -2695,12 +2692,12 @@
     </row>
     <row r="18" spans="1:27" s="15" customFormat="1" ht="14.25" customHeight="1">
       <c r="A18" s="20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="29"/>
       <c r="C18" s="29"/>
       <c r="D18" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="29"/>
       <c r="F18" s="30"/>
@@ -2731,7 +2728,7 @@
       <c r="B19" s="30"/>
       <c r="C19" s="30"/>
       <c r="D19" s="20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E19" s="30"/>
       <c r="F19" s="29"/>
@@ -2847,10 +2844,10 @@
         <v>13</v>
       </c>
       <c r="N1" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="O1" s="26" t="s">
         <v>102</v>
-      </c>
-      <c r="O1" s="26" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15">
@@ -2891,13 +2888,13 @@
         <v>12</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="P2" s="3"/>
     </row>

</xml_diff>